<commit_message>
feat: data-driven baking window assignment per bakery profile
- Replaced static template schedule with peak-detection algorithm:
  hourly forecast -> cluster peaks -> centroid-to-window mapping
- Added parse_comments_sheet(): reads dough group / kratnost / two-day
  flags from the comments sheet added to all templates
- Defrost placed at last window (end of shift), sized from next-day
  early hours; excluded from today bake coverage
- Group-based window assignment: all SKUs in same dough group share
  windows; fallback to template pre-filled schedule when no profile
- Added comments sheet to baking_plan_template.xlsx and individual
  bakery templates (20, 21, 22)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/forecast_embedded/app/assets/baking_plan_individual/22_sibirskiy_trakt_25.xlsx
+++ b/apps/forecast_embedded/app/assets/baking_plan_individual/22_sibirskiy_trakt_25.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="от 4 млн" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="комментарии" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -663,7 +664,7 @@
     <col width="10.6640625" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="15.88671875" customWidth="1" min="11" max="11"/>
-    <col hidden="1" min="13" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1">
@@ -2709,8 +2710,6 @@
       <c r="J56" s="17" t="n"/>
       <c r="K56" s="17" t="n"/>
     </row>
-    <row r="57"/>
-    <row r="58"/>
     <row r="59">
       <c r="A59" s="47" t="n"/>
       <c r="B59" s="48" t="inlineStr">
@@ -2719,8 +2718,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="B62" s="49" t="inlineStr">
         <is>
@@ -2756,8 +2753,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
-    <row r="68"/>
     <row r="69">
       <c r="B69" s="49" t="inlineStr">
         <is>
@@ -2801,4 +2796,1644 @@
   <pageMargins left="0.2362204724409449" right="0.2362204724409449" top="0.3543307086614174" bottom="0.3543307086614174" header="0.3149606299212598" footer="0.3149606299212598"/>
   <pageSetup orientation="landscape" paperSize="9" scale="92" fitToHeight="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M114"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Группировка по тестам</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Тесто на треугольники</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>кратность выпуска</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Треугольник курица безд</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Треугольник говядина безд</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Треугольник острый</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Тесто на элеш</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Элеш с курицей</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Пирог Ханский</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Тесто сдобное</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Вак-бэлиш</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Жар пицца с курицей</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Пицца с колбасой</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Пирожок с горбушей</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Конвертик курица</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Пирожок с картошкой</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Пицца закрытая</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>мини Бургер с котлетой</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Сосиска в тесте</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Беккен капуста</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Сосиска под шубой</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Киш грибы курица</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Шафран творог</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ватрушка</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Пирожок яблоко</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Маковка</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Яблочный</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Пирог с черносливом и грец орехом</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Капустный</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Капуста и мясо</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Горбуша саго</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Замороженные полуфабрикаты (ничего с ними не делаем)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Круассан миндальный</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Круассан с малиной</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Круассан с шоколадом</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Тесто песочное</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Киш курица</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Корзинка ягодная</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Сметанник мини</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Губадия мини</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>двухдневка</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Трехслойник НОВЫЙ</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>двухдневка</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Клубника и банан НОВЫЙ</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>двухдневка</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Тропический</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>двухдневка</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Сметанник</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Губадия</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>двухдневка</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Пирог с Манго</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Пирог с киви</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Пирог Ягодный</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Сметанник маковый</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Жар Киш курица</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Жар Киш грибы курица</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Фастфуд</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Основа коржи покупные</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Помощник пекаря</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ЖарПицца с салями</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Помощник пекаря</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ЖарПицца Пикантная</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Помощник пекаря</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>ЖарПицца Оригинальная</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Основа булочка бейгл покупная</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Помощник пекаря</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Бейгл курица</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Основа тартилья сырная покупная</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Помощник пекаря</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Жар ролл с ветчиной</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Помощник пекаря</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Жар ролл с крабом</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Основа чиабатта покупная</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Помощник пекаря</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Сэндвич Мюнхенский</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Помощник пекаря</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Сэндвич курица</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Основа рис для суши мицукан (проект роллы пекарни)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Они гири с креветкой</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Они гири с курицей</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Они гири с лососем</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Поке с креветкой</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Поке с лососем</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Роллы Вулкан с курицей</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Роллы Запеченные с креветкой</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Роллы запеченные с курицей</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Роллы лосось запеч</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Роллы Филадельфия</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Роллы Вулкан в тубусе</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Роллы Филадельфия в тубусе</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сушист </t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Мексиканский ролл</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Хот доги по запросу клиента</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Помощник продавца</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Хот-дог Баварский говяжий</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Помощник продавца</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Хот-дог Баварский куриный</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Помощник продавца</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Хот-дог Датский говяжий</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Помощник продавца</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Хот-дог Датский куриный</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>по запросу</t>
+        </is>
+      </c>
+    </row>
+    <row r="85"/>
+    <row r="86">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Основа выпекается в пекарне</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Помощник пекаря</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Кыстыбый П</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Индивидуальные теста</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Сочень</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>10</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>двухдневка</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Королевская ватрушка</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Пекарь</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Кексовый манго</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>двухдневка</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Проект пиццы большой</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Пицца Маргарита П (целая)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>1 (в ней 6 кусков)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Пицца Маргарита кусок</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Пицца с салями П</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>1 (в ней 6 кусков)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Пицца с салями кусок</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Пицца Мясная</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>1 (в ней 6 кусков)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Пицца Мясная кусок</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="99"/>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Нормативы по штату ПЕКАРЕЙ с учетом розничных цен на январь 2026г</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Выработка в руб/месяц</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1 пекарь</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>1,5 пекаря</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>2 пекаря</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>3 пекаря</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>4 пекаря</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Мелкоштучка (69)</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1063389.811642685</v>
+      </c>
+      <c r="C102" t="n">
+        <v>1711200</v>
+      </c>
+      <c r="D102" t="n">
+        <v>2058173.828985841</v>
+      </c>
+      <c r="E102" t="n">
+        <v>3087260.743478761</v>
+      </c>
+      <c r="F102" t="n">
+        <v>4140000</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Пироги (277)</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>581890.4445712685</v>
+      </c>
+      <c r="C103" t="n">
+        <v>872550</v>
+      </c>
+      <c r="D103" t="n">
+        <v>1163400</v>
+      </c>
+      <c r="E103" t="n">
+        <v>1745100</v>
+      </c>
+      <c r="F103" t="n">
+        <v>2326800</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Итого пироги и мелкоштучка</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>1645280.256213953</v>
+      </c>
+      <c r="C104" t="n">
+        <v>2583750</v>
+      </c>
+      <c r="D104" t="n">
+        <v>3221573.828985841</v>
+      </c>
+      <c r="E104" t="n">
+        <v>4832360.743478761</v>
+      </c>
+      <c r="F104" t="n">
+        <v>6466800</v>
+      </c>
+    </row>
+    <row r="105"/>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Выработка в шт/день</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1 пекарь</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>1,5 пекаря</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>2 пекаря</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>3 пекаря</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>4 пекаря</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Мелкоштучка</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>500</v>
+      </c>
+      <c r="C107" t="n">
+        <v>800</v>
+      </c>
+      <c r="D107" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E107" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F107" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Пироги</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>70</v>
+      </c>
+      <c r="C108" t="n">
+        <v>100</v>
+      </c>
+      <c r="D108" t="n">
+        <v>140</v>
+      </c>
+      <c r="E108" t="n">
+        <v>210</v>
+      </c>
+      <c r="F108" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Итого пироги и мелкоштучка</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>600</v>
+      </c>
+      <c r="C109" t="n">
+        <v>900</v>
+      </c>
+      <c r="D109" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E109" t="n">
+        <v>1710</v>
+      </c>
+      <c r="F109" t="n">
+        <v>2280</v>
+      </c>
+    </row>
+    <row r="110"/>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Выработка в шт/месяц</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1 пекарь</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>1,5 пекаря</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>2 пекаря</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>3 пекаря</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>4 пекаря</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Мелкоштучка</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>15500</v>
+      </c>
+      <c r="C112" t="n">
+        <v>24800</v>
+      </c>
+      <c r="D112" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E112" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F112" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Пироги</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>2100</v>
+      </c>
+      <c r="C113" t="n">
+        <v>3150</v>
+      </c>
+      <c r="D113" t="n">
+        <v>4200</v>
+      </c>
+      <c r="E113" t="n">
+        <v>6300</v>
+      </c>
+      <c r="F113" t="n">
+        <v>8400</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Итого пироги и мелкоштучка</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>17600</v>
+      </c>
+      <c r="C114" t="n">
+        <v>27950</v>
+      </c>
+      <c r="D114" t="n">
+        <v>34200</v>
+      </c>
+      <c r="E114" t="n">
+        <v>51300</v>
+      </c>
+      <c r="F114" t="n">
+        <v>68400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>